<commit_message>
docs: :memo: Relleno del excel con la dedicación de horas del sprint WPL
Refs: #542
</commit_message>
<xml_diff>
--- a/docs/Sprint WPL/Entrega/9-WPL-dedication.xlsx
+++ b/docs/Sprint WPL/Entrega/9-WPL-dedication.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uses0.sharepoint.com/sites/ISPP_dvkxr7/Documentos compartidos/General/ENTREGABLE PPL/EV/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uses0.sharepoint.com/sites/ISPP_dvkxr7/Documentos compartidos/General/ENTREGABLE WPL/EV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{876CD675-13DD-4782-8363-D5089FCF8529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A956B201-1E32-47F6-9778-0F2C24731652}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{876CD675-13DD-4782-8363-D5089FCF8529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44160B55-ABB0-42CD-A029-AC23690511AE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{02C8C9D8-2F21-45BA-9A66-91BB45160C54}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{02C8C9D8-2F21-45BA-9A66-91BB45160C54}"/>
   </bookViews>
   <sheets>
     <sheet name="Contribución a los entregables" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
   <si>
     <t>Nombre</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>El compañero Manuel Jesús Benito Merchán no pudo completar sus horas debido a problemas personales, por lo que algunas personas del grupo hicieron algunas pocas horas de más para compensarlo</t>
+  </si>
+  <si>
+    <t>World project launch (#WPL)</t>
   </si>
 </sst>
 </file>
@@ -285,7 +288,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -312,51 +315,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -368,21 +326,6 @@
       </left>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -448,12 +391,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -465,82 +449,79 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -966,7 +947,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30DF89C9-C95E-4402-8344-C5801FC30A20}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
@@ -974,601 +955,673 @@
     <col min="3" max="7" width="10.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="23" t="s">
+      <c r="B1" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="H1" s="31" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="6">
-        <v>1</v>
-      </c>
-      <c r="D2" s="6">
-        <v>1</v>
-      </c>
-      <c r="E2" s="6">
+      <c r="C2" s="29">
+        <v>1</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1</v>
+      </c>
+      <c r="E2" s="29">
         <v>1.05</v>
       </c>
-      <c r="F2" s="6">
-        <v>1</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="F2" s="29">
+        <v>1</v>
+      </c>
+      <c r="G2" s="29">
+        <v>1</v>
+      </c>
+      <c r="H2" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="6">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6">
-        <v>1</v>
-      </c>
-      <c r="E3" s="6">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5">
         <v>1.01</v>
       </c>
-      <c r="F3" s="6">
-        <v>1</v>
-      </c>
-      <c r="G3" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+      <c r="F3" s="5">
+        <v>1</v>
+      </c>
+      <c r="G3" s="5">
+        <v>1</v>
+      </c>
+      <c r="H3" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6">
-        <v>1</v>
-      </c>
-      <c r="D4" s="6">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6">
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
         <v>0.83</v>
       </c>
-      <c r="F4" s="6">
-        <v>1</v>
-      </c>
-      <c r="G4" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="F4" s="5">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5">
+        <v>1</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6">
-        <v>1</v>
-      </c>
-      <c r="E5" s="6">
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
         <v>1.03</v>
       </c>
-      <c r="F5" s="6">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="F5" s="5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1</v>
-      </c>
-      <c r="F6" s="6">
-        <v>1</v>
-      </c>
-      <c r="G6" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="6">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="6">
-        <v>1</v>
-      </c>
-      <c r="F7" s="6">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="6">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6">
+      <c r="C8" s="5">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5">
         <v>1.03</v>
       </c>
-      <c r="F8" s="6">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="F8" s="5">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="6">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="C9" s="5">
+        <v>1</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5">
         <v>1.01</v>
       </c>
-      <c r="F9" s="6">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
+      <c r="F9" s="5">
+        <v>1</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="6">
-        <v>1</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6">
-        <v>1</v>
-      </c>
-      <c r="F10" s="6">
-        <v>1</v>
-      </c>
-      <c r="G10" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
+      <c r="C10" s="5">
+        <v>1</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1</v>
+      </c>
+      <c r="F10" s="5">
+        <v>1</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1</v>
+      </c>
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="6">
-        <v>1</v>
-      </c>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6">
-        <v>1</v>
-      </c>
-      <c r="F11" s="6">
-        <v>1</v>
-      </c>
-      <c r="G11" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
+      <c r="C11" s="5">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="6">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
+      <c r="C12" s="5">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1</v>
+      </c>
+      <c r="F12" s="5">
+        <v>1</v>
+      </c>
+      <c r="G12" s="5">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="6">
-        <v>1</v>
-      </c>
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="6">
-        <v>1</v>
-      </c>
-      <c r="F13" s="6">
-        <v>1</v>
-      </c>
-      <c r="G13" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
+      <c r="C13" s="5">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5">
+        <v>1</v>
+      </c>
+      <c r="F13" s="5">
+        <v>1</v>
+      </c>
+      <c r="G13" s="5">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="6">
-        <v>1</v>
-      </c>
-      <c r="D14" s="6">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6">
-        <v>1</v>
-      </c>
-      <c r="F14" s="6">
-        <v>1</v>
-      </c>
-      <c r="G14" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+      <c r="C14" s="5">
+        <v>1</v>
+      </c>
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1</v>
+      </c>
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="5">
+        <v>1</v>
+      </c>
+      <c r="H14" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="6">
-        <v>1</v>
-      </c>
-      <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6">
-        <v>1</v>
-      </c>
-      <c r="G15" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="8" t="s">
+      <c r="C15" s="5">
+        <v>1</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5">
+        <v>1</v>
+      </c>
+      <c r="H15" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="6">
-        <v>1</v>
-      </c>
-      <c r="D16" s="6">
-        <v>1</v>
-      </c>
-      <c r="E16" s="6">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6">
-        <v>1</v>
-      </c>
-      <c r="G16" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
+      <c r="C16" s="5">
+        <v>1</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5">
+        <v>1</v>
+      </c>
+      <c r="G16" s="5">
+        <v>1</v>
+      </c>
+      <c r="H16" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="6">
-        <v>1</v>
-      </c>
-      <c r="D17" s="6">
-        <v>1</v>
-      </c>
-      <c r="E17" s="6">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6">
-        <v>1</v>
-      </c>
-      <c r="G17" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="8" t="s">
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5">
+        <v>1</v>
+      </c>
+      <c r="G17" s="5">
+        <v>1</v>
+      </c>
+      <c r="H17" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="6">
-        <v>1</v>
-      </c>
-      <c r="D18" s="6">
-        <v>1</v>
-      </c>
-      <c r="E18" s="6">
-        <v>1</v>
-      </c>
-      <c r="F18" s="6">
-        <v>1</v>
-      </c>
-      <c r="G18" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="8" t="s">
+      <c r="C18" s="5">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5">
+        <v>1</v>
+      </c>
+      <c r="G18" s="5">
+        <v>1</v>
+      </c>
+      <c r="H18" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="6">
-        <v>1</v>
-      </c>
-      <c r="D19" s="6">
-        <v>1</v>
-      </c>
-      <c r="E19" s="6">
-        <v>1</v>
-      </c>
-      <c r="F19" s="6">
-        <v>1</v>
-      </c>
-      <c r="G19" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5">
+        <v>1</v>
+      </c>
+      <c r="E19" s="5">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5">
+        <v>1</v>
+      </c>
+      <c r="G19" s="5">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="6">
-        <v>1</v>
-      </c>
-      <c r="D20" s="6">
-        <v>1</v>
-      </c>
-      <c r="E20" s="6">
+      <c r="C20" s="5">
+        <v>1</v>
+      </c>
+      <c r="D20" s="5">
+        <v>1</v>
+      </c>
+      <c r="E20" s="5">
         <v>1.04</v>
       </c>
-      <c r="F20" s="6">
-        <v>1</v>
-      </c>
-      <c r="G20" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="9" t="s">
+      <c r="F20" s="5">
+        <v>1</v>
+      </c>
+      <c r="G20" s="5">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="7">
-        <v>1</v>
-      </c>
-      <c r="D21" s="7">
-        <v>1</v>
-      </c>
-      <c r="E21" s="7">
-        <v>1</v>
-      </c>
-      <c r="F21" s="7">
-        <v>1</v>
-      </c>
-      <c r="G21" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+      <c r="C21" s="26">
+        <v>1</v>
+      </c>
+      <c r="D21" s="26">
+        <v>1</v>
+      </c>
+      <c r="E21" s="26">
+        <v>1</v>
+      </c>
+      <c r="F21" s="26">
+        <v>1</v>
+      </c>
+      <c r="G21" s="26">
+        <v>1</v>
+      </c>
+      <c r="H21" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="10">
         <f>COUNTA(A2:A21)</f>
         <v>20</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="14"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="16">
+      <c r="B23" s="28"/>
+      <c r="C23" s="12">
         <f>SUM(C2:C21)/$B$22</f>
         <v>1</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="12">
         <f>SUM(D2:D21)/$B$22</f>
         <v>1</v>
       </c>
-      <c r="E23" s="16">
+      <c r="E23" s="12">
         <f>SUM(E2:E21)/$B$22</f>
         <v>1</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="12">
         <f>SUM(F2:F21)/$B$22</f>
         <v>1</v>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="12">
         <f>SUM(G2:G21)/$B$22</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="12" t="s">
+      <c r="H23" s="13">
+        <f>SUM(H2:H21)/$B$22</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="19">
+      <c r="B24" s="14"/>
+      <c r="C24" s="15">
         <f>1-C23</f>
         <v>0</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="15">
         <f t="shared" ref="D24:G24" si="0">1-D23</f>
         <v>0</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G24" s="20">
+      <c r="G24" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="29" t="s">
+      <c r="H24" s="16">
+        <f t="shared" ref="H24" si="1">1-H23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="14"/>
-    </row>
-    <row r="28" spans="1:7" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="30"/>
-      <c r="B28" s="25" t="s">
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+    </row>
+    <row r="28" spans="1:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="23"/>
+      <c r="B28" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="26"/>
-    </row>
-    <row r="29" spans="1:7" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="30"/>
-      <c r="B29" s="25" t="s">
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="19"/>
+    </row>
+    <row r="29" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="23"/>
+      <c r="B29" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="26"/>
-    </row>
-    <row r="30" spans="1:7" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="31"/>
-      <c r="B30" s="27" t="s">
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="19"/>
+    </row>
+    <row r="30" spans="1:8" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="24"/>
+      <c r="B30" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="28"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="21"/>
     </row>
     <row r="33" spans="4:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="D33" s="3"/>
@@ -1580,7 +1633,7 @@
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="A27:A30"/>
   </mergeCells>
-  <conditionalFormatting sqref="C23:G23">
+  <conditionalFormatting sqref="C23:H23">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>1</formula>
     </cfRule>
@@ -1594,7 +1647,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24:G24">
+  <conditionalFormatting sqref="C24:H24">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>""</formula>
     </cfRule>
@@ -1645,13 +1698,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1680,15 +1733,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007CF12EDFE4592B42B175CC2F30328DE8" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="2d6dd0d3c599ad09928ee51439f12a6b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e65dd739-d64f-453c-9fd1-fed4e9613ba5" xmlns:ns3="fdf96737-606d-4cc9-9eb0-41eef5b03e89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="92a042fa933df5bdb65e6461d477892f" ns2:_="" ns3:_="">
     <xsd:import namespace="e65dd739-d64f-453c-9fd1-fed4e9613ba5"/>
@@ -1889,6 +1933,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1901,14 +1954,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCB68768-760F-4B2D-AD9E-DC7F1895DB84}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1927,6 +1972,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D0D844A-E87E-42E2-B155-132CABE67861}">
   <ds:schemaRefs>

</xml_diff>